<commit_message>
Sheet 2/10 接入 ShopperTrak 來客數（人流）
- 新增 shoppertrak_traffic.py：Playwright 無頭瀏覽器登入 SSO（比照人流插件
  填表邏輯，讀 sessionStorage authToken/tenantId），requests 查 kpis API。
  EPB shop_id → siteId 對照、token 快取、本機帳密與編制人數設定。
- fill_sheet2/fill_sheet10 新增選用參數 traffic/emp_count：
  填 來客數、提袋率(=成交筆數/來客數)、人均產值(=總營業額/編制人數)。
- server.py：load_traffic 一次登入抓 7 期間，失敗則略過、其餘照常產生；
  新增 /api/shoppertrak/status、/api/shoppertrak/credentials、/api/config；
  _run_job 改傳完整 payload（順帶修正 yoyEnd 未傳入的問題）。
- 前端新增來客數帳密設定區與編制人數欄位（記住上次輸入）。
- 啟動腳本自動安裝 requests / playwright / chromium；local_config.json 加入 .gitignore。
- 修正週報模板 Sheet 2 人均產值/來客數兩列的科學記號格式 → #,##0。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/週報模板.xlsx
+++ b/週報模板.xlsx
@@ -421,7 +421,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -755,6 +755,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -4642,28 +4648,28 @@
           <t>人均產值</t>
         </is>
       </c>
-      <c r="B31" s="37" t="n"/>
-      <c r="C31" s="37" t="n"/>
-      <c r="D31" s="38" t="n">
+      <c r="B31" s="115" t="n"/>
+      <c r="C31" s="115" t="n"/>
+      <c r="D31" s="116" t="n">
         <v>100000</v>
       </c>
       <c r="E31" s="31" t="n">
         <v>0.18</v>
       </c>
-      <c r="F31" s="37" t="n"/>
+      <c r="F31" s="115" t="n"/>
       <c r="G31" s="32" t="n"/>
       <c r="H31" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="I31" s="37" t="n"/>
-      <c r="J31" s="38" t="n">
+      <c r="I31" s="115" t="n"/>
+      <c r="J31" s="116" t="n">
         <v>-800000</v>
       </c>
       <c r="K31" s="31" t="n">
         <v>-0.32</v>
       </c>
-      <c r="L31" s="37" t="n"/>
-      <c r="M31" s="38" t="n">
+      <c r="L31" s="115" t="n"/>
+      <c r="M31" s="116" t="n">
         <v>300000</v>
       </c>
       <c r="N31" s="31" t="n">
@@ -4676,15 +4682,15 @@
           <t>來客數</t>
         </is>
       </c>
-      <c r="B32" s="37" t="n"/>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="38" t="n">
+      <c r="B32" s="115" t="n"/>
+      <c r="C32" s="115" t="n"/>
+      <c r="D32" s="116" t="n">
         <v>-200</v>
       </c>
       <c r="E32" s="31" t="n">
         <v>-0.14</v>
       </c>
-      <c r="F32" s="37" t="n"/>
+      <c r="F32" s="115" t="n"/>
       <c r="G32" s="30" t="n">
         <v>0</v>
       </c>
@@ -4692,14 +4698,14 @@
         <v>0</v>
       </c>
       <c r="I32" s="29" t="n"/>
-      <c r="J32" s="38" t="n">
+      <c r="J32" s="116" t="n">
         <v>-500</v>
       </c>
       <c r="K32" s="31" t="n">
         <v>-0.08</v>
       </c>
-      <c r="L32" s="37" t="n"/>
-      <c r="M32" s="38" t="n">
+      <c r="L32" s="115" t="n"/>
+      <c r="M32" s="116" t="n">
         <v>-900</v>
       </c>
       <c r="N32" s="31" t="n">

</xml_diff>